<commit_message>
Cambios en la interfaz
</commit_message>
<xml_diff>
--- a/Informe_Final_Combinado.xlsx
+++ b/Informe_Final_Combinado.xlsx
@@ -7,8 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Mortalidad" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Lluvia" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Mortalidad_por_Mes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Lluvia_por_Mes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Localidades" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Actor_Vial" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -698,4 +700,306 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>LOCALIDAD</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>casos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Kennedy</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Engativá</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Suba</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ciudad Bolívar</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Fontibón</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bosa</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Puente Aranda</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Usaquén</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tunjuelito</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Usme</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Sin dato</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>San Cristóbal</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Rafael Uribe Uribe</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Los Mártires</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Teusaquillo</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Barrios Unidos</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Antonio Nariño</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Chapinero</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>La Candelaria</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Sumapaz</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>CONDICION_DE_LA_VICTIMA_AT_</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>casos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Conductor</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5890</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Peatón</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5310</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pasajero</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1112</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sin información</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>